<commit_message>
edit size of char
edit size and type of char, add in ai-edited "dev notes"
</commit_message>
<xml_diff>
--- a/Database 1.xlsx
+++ b/Database 1.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Charlie\Non Puriel\Adress-Shack\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A261A577-2A4D-4EF5-B1E6-C341028E30A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7017824F-7220-4F73-A929-5C805913F6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sample Data 2" sheetId="7" r:id="rId1"/>
-    <sheet name="SampleData" sheetId="2" r:id="rId2"/>
-    <sheet name="Address Book" sheetId="1" r:id="rId3"/>
-    <sheet name="Snacks" sheetId="4" r:id="rId4"/>
-    <sheet name="Vending" sheetId="5" r:id="rId5"/>
-    <sheet name="Sales" sheetId="6" r:id="rId6"/>
+    <sheet name="Dev Notes" sheetId="8" r:id="rId1"/>
+    <sheet name="Sample Data 2" sheetId="7" r:id="rId2"/>
+    <sheet name="SampleData" sheetId="2" r:id="rId3"/>
+    <sheet name="Address Book" sheetId="1" r:id="rId4"/>
+    <sheet name="Snacks" sheetId="4" r:id="rId5"/>
+    <sheet name="Vending" sheetId="5" r:id="rId6"/>
+    <sheet name="Sales" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,7 +45,121 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="148">
+  <si>
+    <t>📋 Snack Shack - Dev Notes</t>
+  </si>
+  <si>
+    <t>Track implemented concepts, schema decisions, and design rationale</t>
+  </si>
+  <si>
+    <t>✅ Implemented Concepts</t>
+  </si>
+  <si>
+    <t>Concept</t>
+  </si>
+  <si>
+    <t>Date Implemented</t>
+  </si>
+  <si>
+    <t>Sheet/Location</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>CSV to Spreadsheet parsing</t>
+  </si>
+  <si>
+    <t>Sample Data 2</t>
+  </si>
+  <si>
+    <t>Split comma-separated values into columns A-E</t>
+  </si>
+  <si>
+    <t>🗄️ Schema Decisions</t>
+  </si>
+  <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Decision</t>
+  </si>
+  <si>
+    <t>Rationale</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Snacks</t>
+  </si>
+  <si>
+    <t>SnackID</t>
+  </si>
+  <si>
+    <t>1-based indexing</t>
+  </si>
+  <si>
+    <t>SQL identity convention, human-readable</t>
+  </si>
+  <si>
+    <t>Image Path</t>
+  </si>
+  <si>
+    <t>Store filename only (no ext?)</t>
+  </si>
+  <si>
+    <t>TBD: char(10) constraint, reconstruct path in app</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>smallmoney</t>
+  </si>
+  <si>
+    <t>Sufficient precision for snack prices</t>
+  </si>
+  <si>
+    <t>❓ Open Questions / To-Do</t>
+  </si>
+  <si>
+    <t>Question/Task</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Resolution</t>
+  </si>
+  <si>
+    <t>Image path strategy: extension handling</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Options: strip ext + standardize .jpg, or dynamic detection</t>
+  </si>
+  <si>
+    <t>Valid column purpose</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>Path length validation testing</t>
+  </si>
+  <si>
+    <t>Vending/Sales table schema</t>
+  </si>
+  <si>
+    <t>Not Started</t>
+  </si>
   <si>
     <t>Test</t>
   </si>
@@ -152,9 +267,6 @@
   </si>
   <si>
     <t>Type</t>
-  </si>
-  <si>
-    <t>Notes</t>
   </si>
   <si>
     <t>Validated</t>
@@ -311,30 +423,18 @@
     <t>bit</t>
   </si>
   <si>
-    <t>SnackID</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
-    <t>Price</t>
-  </si>
-  <si>
     <t>Quantity On Hand</t>
   </si>
   <si>
-    <t>Image Path</t>
-  </si>
-  <si>
     <t>Column1</t>
   </si>
   <si>
     <t>Valid</t>
   </si>
   <si>
-    <t>Field</t>
-  </si>
-  <si>
     <t>C# Data Type</t>
   </si>
   <si>
@@ -356,7 +456,7 @@
     <t>airheads.jpg</t>
   </si>
   <si>
-    <t>char(30)</t>
+    <t>varchar(30)</t>
   </si>
   <si>
     <t>name of the snack</t>
@@ -365,9 +465,6 @@
     <t>float</t>
   </si>
   <si>
-    <t>smallmoney</t>
-  </si>
-  <si>
     <t>price of snack</t>
   </si>
   <si>
@@ -381,6 +478,9 @@
   </si>
   <si>
     <t>quantity of snack</t>
+  </si>
+  <si>
+    <t>varchar(15)</t>
   </si>
   <si>
     <t>path of image</t>
@@ -399,7 +499,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -421,13 +521,76 @@
       <name val="Aptos Narrow"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF666666"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF808080"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -443,7 +606,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -455,6 +618,14 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -517,7 +688,7 @@
     <tableColumn id="4" xr3:uid="{01AF8722-0E57-4D45-8F72-AD068B958406}" name="Image Path"/>
     <tableColumn id="6" xr3:uid="{85B6F931-9CA9-4FF4-9FB1-406FC9E56BA6}" name="Column1"/>
     <tableColumn id="7" xr3:uid="{AEC76C43-8C35-4A51-B34A-C477D5C7F079}" name="Valid" dataDxfId="0">
-      <calculatedColumnFormula>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -820,6 +991,186 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C3DB4FA-A95C-4424-BD58-265C1159E376}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="41.85546875" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" customWidth="1"/>
+    <col min="3" max="3" width="34.28515625" customWidth="1"/>
+    <col min="4" max="4" width="53.28515625" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="21">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.75">
+      <c r="A4" s="9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="12">
+        <v>46153</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15.75">
+      <c r="A9" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="12">
+        <v>46153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="12">
+        <v>46153</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" s="12">
+        <v>46153</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15.75">
+      <c r="A16" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="11"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ECEA5BB-8E4E-42E6-AD28-A777D9306799}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -834,7 +1185,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="B1">
         <v>0.05</v>
@@ -843,7 +1194,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="E1">
         <v>0</v>
@@ -851,7 +1202,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>7.0000000000000007E-2</v>
@@ -860,7 +1211,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -868,7 +1219,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B3">
         <v>0.7</v>
@@ -877,7 +1228,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="E3">
         <v>2</v>
@@ -885,7 +1236,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="B4">
         <v>0.05</v>
@@ -894,7 +1245,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -902,7 +1253,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="B5">
         <v>7.0000000000000007E-2</v>
@@ -911,7 +1262,7 @@
         <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -919,7 +1270,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B6">
         <v>7.0000000000000007E-2</v>
@@ -928,7 +1279,7 @@
         <v>97</v>
       </c>
       <c r="D6" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -936,7 +1287,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B7">
         <v>0.08</v>
@@ -945,7 +1296,7 @@
         <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="E7">
         <v>6</v>
@@ -953,7 +1304,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B8">
         <v>7.0000000000000007E-2</v>
@@ -962,7 +1313,7 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>9</v>
+        <v>47</v>
       </c>
       <c r="E8">
         <v>7</v>
@@ -970,7 +1321,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B9">
         <v>7.0000000000000007E-2</v>
@@ -979,7 +1330,7 @@
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="E9">
         <v>8</v>
@@ -987,7 +1338,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="B10">
         <v>0.05</v>
@@ -996,7 +1347,7 @@
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="E10">
         <v>9</v>
@@ -1004,7 +1355,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="B11">
         <v>0.05</v>
@@ -1013,7 +1364,7 @@
         <v>0</v>
       </c>
       <c r="D11" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -1024,7 +1375,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F28EEB29-88E9-4F91-A919-2DF8C70E2648}">
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1039,22 +1390,22 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C1">
         <v>1</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="E1" t="b">
         <v>1</v>
       </c>
       <c r="F1" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="G1">
         <v>1</v>
@@ -1062,22 +1413,22 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="G2">
         <v>2</v>
@@ -1085,22 +1436,22 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C3">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="G3">
         <v>3</v>
@@ -1108,10 +1459,10 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="D4">
         <v>11</v>
@@ -1128,22 +1479,22 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="G5">
         <v>5</v>
@@ -1151,22 +1502,22 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="G6">
         <v>6</v>
@@ -1174,13 +1525,13 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1189,7 +1540,7 @@
         <v>0</v>
       </c>
       <c r="F7" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="G7">
         <v>7</v>
@@ -1197,13 +1548,13 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1212,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="G8">
         <v>8</v>
@@ -1220,10 +1571,10 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>57</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1235,7 +1586,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="G9">
         <v>9</v>
@@ -1266,10 +1617,10 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1281,7 +1632,7 @@
         <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="G11">
         <v>11</v>
@@ -1289,22 +1640,22 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="C12">
         <v>1234567891</v>
       </c>
       <c r="D12" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>23</v>
+        <v>61</v>
       </c>
       <c r="G12">
         <v>12</v>
@@ -1312,42 +1663,42 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C13">
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="G14">
         <v>14</v>
@@ -1355,7 +1706,7 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -1366,7 +1717,7 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -1377,7 +1728,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -1388,22 +1739,22 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C18">
         <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>24</v>
+        <v>62</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>28</v>
+        <v>66</v>
       </c>
       <c r="G18">
         <v>18</v>
@@ -1426,7 +1777,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="G19">
         <v>19</v>
@@ -1434,22 +1785,22 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="B20" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
       <c r="D20" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="G20">
         <v>20</v>
@@ -1460,7 +1811,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AC24"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1480,37 +1831,37 @@
   <sheetData>
     <row r="1" spans="1:15" ht="30">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>68</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>70</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="G1" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="J1" t="s">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="K1" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="30">
@@ -1519,32 +1870,32 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="D2">
         <v>2345678901</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="I2" s="3"/>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="K2" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>46</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="45">
@@ -1553,32 +1904,32 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="D3">
         <v>2811111111</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="F3">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>50</v>
+        <v>87</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="K3" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>51</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -1587,32 +1938,32 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="D4">
         <v>2209371286</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>53</v>
+        <v>90</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="K4" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>54</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="30">
@@ -1621,35 +1972,35 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="D5">
         <v>9876111121</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>57</v>
+        <v>94</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="K5" t="s">
-        <v>58</v>
+        <v>95</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>59</v>
+        <v>96</v>
       </c>
       <c r="O5" t="s">
-        <v>60</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -1658,29 +2009,29 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="C6" t="s">
-        <v>62</v>
+        <v>99</v>
       </c>
       <c r="D6">
         <v>1291821021</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" t="s">
-        <v>36</v>
+        <v>6</v>
       </c>
       <c r="K6" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>65</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -1689,16 +2040,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>99</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>98</v>
       </c>
       <c r="D7">
         <v>1234543201</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>66</v>
+        <v>103</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -1710,22 +2061,22 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>105</v>
       </c>
       <c r="D8">
         <v>1234562311</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>69</v>
+        <v>106</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -1734,22 +2085,22 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>108</v>
       </c>
       <c r="D9">
         <v>1234567812</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>72</v>
+        <v>109</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -1758,22 +2109,22 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="D10" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10" t="s">
-        <v>77</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1782,38 +2133,38 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>78</v>
+        <v>115</v>
       </c>
       <c r="C11" t="s">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="D11">
         <v>2312121212</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>81</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:29">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="1:29">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>120</v>
       </c>
       <c r="B18" t="s">
-        <v>83</v>
+        <v>120</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>120</v>
       </c>
       <c r="D18">
         <v>10</v>
@@ -1824,43 +2175,43 @@
     </row>
     <row r="19" spans="1:29">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>121</v>
       </c>
       <c r="B19" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="C19" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="D19" t="s">
-        <v>86</v>
+        <v>123</v>
       </c>
       <c r="E19" t="s">
-        <v>85</v>
+        <v>122</v>
       </c>
       <c r="F19" t="s">
-        <v>87</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23" spans="1:29">
       <c r="P23" s="1"/>
       <c r="W23" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="X23" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="Y23">
         <v>1</v>
       </c>
       <c r="Z23" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="AA23" t="b">
         <v>0</v>
       </c>
       <c r="AB23" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="AC23">
         <v>2</v>
@@ -1868,22 +2219,22 @@
     </row>
     <row r="24" spans="1:29">
       <c r="W24" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="X24" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="Y24">
         <v>2</v>
       </c>
       <c r="Z24" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="AA24" t="b">
         <v>1</v>
       </c>
       <c r="AB24" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="AC24">
         <v>3</v>
@@ -1912,7 +2263,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7BC218-E894-43DE-BEC3-7A8A07868B41}">
   <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1929,37 +2280,37 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" t="s">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>91</v>
+        <v>126</v>
       </c>
       <c r="E1" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>93</v>
+        <v>127</v>
       </c>
       <c r="G1" t="s">
-        <v>94</v>
+        <v>128</v>
       </c>
       <c r="J1" t="s">
-        <v>95</v>
+        <v>12</v>
       </c>
       <c r="K1" t="s">
-        <v>96</v>
+        <v>129</v>
       </c>
       <c r="L1" t="s">
-        <v>97</v>
+        <v>130</v>
       </c>
       <c r="M1" t="s">
-        <v>98</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -1968,7 +2319,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="C2" s="4">
         <v>0.05</v>
@@ -1977,23 +2328,23 @@
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="G2" t="b">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="K2" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="L2" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="M2" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2002,7 +2353,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C3" s="4">
         <v>7.0000000000000007E-2</v>
@@ -2011,23 +2362,23 @@
         <v>1</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G3" t="str">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
-        <v>FALSE 12</v>
+        <v>135</v>
+      </c>
+      <c r="G3" t="b">
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
       <c r="K3" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="L3" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="M3" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2036,7 +2387,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C4" s="4">
         <v>0.7</v>
@@ -2045,23 +2396,23 @@
         <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="G4" t="b">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>90</v>
+        <v>23</v>
       </c>
       <c r="K4" t="s">
-        <v>105</v>
+        <v>138</v>
       </c>
       <c r="L4" t="s">
-        <v>106</v>
+        <v>24</v>
       </c>
       <c r="M4" t="s">
-        <v>107</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -2070,7 +2421,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="C5" s="4">
         <v>0.05</v>
@@ -2079,23 +2430,23 @@
         <v>0</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="G5" t="str">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
-        <v>FALSE 12</v>
+        <v>140</v>
+      </c>
+      <c r="G5" t="b">
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="K5" t="s">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="L5" t="s">
-        <v>110</v>
+        <v>142</v>
       </c>
       <c r="M5" t="s">
-        <v>111</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2104,7 +2455,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="C6" s="4">
         <v>7.0000000000000007E-2</v>
@@ -2113,23 +2464,23 @@
         <v>33</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G6" s="5" t="str">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
-        <v>FALSE 12</v>
+        <v>135</v>
+      </c>
+      <c r="G6" s="5" t="b">
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="K6" t="s">
-        <v>64</v>
+        <v>101</v>
       </c>
       <c r="L6" t="s">
-        <v>86</v>
+        <v>144</v>
       </c>
       <c r="M6" t="s">
-        <v>112</v>
+        <v>145</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2138,7 +2489,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="C7" s="4">
         <v>7.0000000000000007E-2</v>
@@ -2147,14 +2498,14 @@
         <v>97</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G7" s="5" t="str">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
-        <v>FALSE 12</v>
+        <v>135</v>
+      </c>
+      <c r="G7" s="5" t="b">
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <v>1</v>
       </c>
       <c r="L7">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -2163,7 +2514,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="C8" s="4">
         <v>0.08</v>
@@ -2172,11 +2523,11 @@
         <v>4</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="G8" s="5" t="str">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
-        <v>FALSE 13</v>
+        <v>146</v>
+      </c>
+      <c r="G8" s="5" t="b">
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2185,7 +2536,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C9" s="4">
         <v>7.0000000000000007E-2</v>
@@ -2194,11 +2545,11 @@
         <v>1</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="G9" s="5" t="str">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
-        <v>FALSE 13</v>
+        <v>146</v>
+      </c>
+      <c r="G9" s="5" t="b">
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2207,7 +2558,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="C10" s="4">
         <v>7.0000000000000007E-2</v>
@@ -2216,11 +2567,11 @@
         <v>2</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="G10" s="5" t="str">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
-        <v>FALSE 14</v>
+        <v>147</v>
+      </c>
+      <c r="G10" s="5" t="b">
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -2229,7 +2580,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="C11" s="4">
         <v>0.05</v>
@@ -2238,10 +2589,10 @@
         <v>2</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="G11" s="5" t="b">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
         <v>1</v>
       </c>
     </row>
@@ -2251,7 +2602,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="C12" s="4">
         <v>0.05</v>
@@ -2260,11 +2611,11 @@
         <v>0</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G12" s="5" t="str">
-        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE()," ",LEN(Table2[[#This Row],[Image Path]])))</f>
-        <v>FALSE 12</v>
+        <v>135</v>
+      </c>
+      <c r="G12" s="5" t="b">
+        <f>IF(NOT(LEN(Table2[[#This Row],[Image Path]])&gt;$L$7),TRUE(),_xlfn.CONCAT(FALSE(),": ",LEN(Table2[[#This Row],[Image Path]])))</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2275,7 +2626,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E27DB38-9B86-476F-ADB3-257C50139E20}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2284,7 +2635,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1932462C-482C-40F7-8C16-E10683B0C6A3}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>